<commit_message>
Prepare accounting engine releases and the MCP dependency update
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A24246-3926-4A7F-825D-2E36F977E904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D51E66-9FFA-403F-A95E-7504D3D1AF07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.1.6. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.1.7. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1222,7 +1222,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.6</t>
+    <t>0.1.7</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -1279,7 +1279,7 @@
     <t>2023-24 licence</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20326</t>
+    <t>Excel 16.0 build 20430</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Prepare accounting engine release candidates (#158)
Prepare the component versions and workbook stamps. Local component gates and the complete hosted matrix pass. Publish the three engine prerequisites before completing the standalone MCP release checks.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A24246-3926-4A7F-825D-2E36F977E904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D51E66-9FFA-403F-A95E-7504D3D1AF07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.1.6. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.1.7. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1222,7 +1222,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.6</t>
+    <t>0.1.7</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -1279,7 +1279,7 @@
     <t>2023-24 licence</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20326</t>
+    <t>Excel 16.0 build 20430</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Make refused Division 7A repayments drive REVIEW and close four benchmark workbook review gaps
- div7a-loan-review workbook: a REFUSED repayment row now drives the overall status to REVIEW, matching the engine's attention rule, with its reason and the not-a-breach warning retained. Start Here and the workbook README say so.
- ato-benchmark-compare workbook: tblPnl carries a normalised Key column; the bucket lookup matches on an equality array instead of MATCH's wildcard text form; the bucket check counts unrecognised buckets as well as blank ones; the suggested-mapping count trims and lowercases Source; the P&L duplicate check reads the normalised keys.
- Both workbooks are rebuilt through desktop Excel with fresh cached values.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D51E66-9FFA-403F-A95E-7504D3D1AF07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE72EBA-8DC4-479A-968A-F3AF34DAF2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5124" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5125" uniqueCount="414">
   <si>
     <t>ATO small business benchmark comparison</t>
   </si>
@@ -82,6 +82,9 @@
     <t>Sample</t>
   </si>
   <si>
+    <t>Key</t>
+  </si>
+  <si>
     <t>Sales - bread and rolls</t>
   </si>
   <si>
@@ -169,9 +172,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Key</t>
-  </si>
-  <si>
     <t>turnover</t>
   </si>
   <si>
@@ -1177,7 +1177,7 @@
     <t>Example account</t>
   </si>
   <si>
-    <t>Every P&amp;L account has a bucket</t>
+    <t>Every P&amp;L account has a recognised bucket</t>
   </si>
   <si>
     <t>No mapping is still suggested</t>
@@ -1446,18 +1446,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblPnl" displayName="tblPnl" ref="A1:E28">
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblPnl" displayName="tblPnl" ref="A1:F28">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Account"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Amount"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Bucket">
-      <calculatedColumnFormula>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Guard">
       <calculatedColumnFormula>IF(OR(_xlfn.ISFORMULA(tblPnl[[#This Row],[Account]]),_xlfn.ISFORMULA(tblPnl[[#This Row],[Amount]]),AND(tblPnl[[#This Row],[Account]]&lt;&gt;"",NOT(ISNUMBER(tblPnl[[#This Row],[Amount]])))),1,0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Sample">
       <calculatedColumnFormula>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Key">
+      <calculatedColumnFormula>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1861,7 +1864,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1869,7 +1872,7 @@
     <col min="3" max="3" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1885,16 +1888,19 @@
       <c r="E1" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="7">
         <v>520000</v>
       </c>
       <c r="C2" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>turnover</v>
       </c>
       <c r="D2" s="8">
@@ -1905,16 +1911,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>sales - bread and rolls</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="7">
         <v>330000</v>
       </c>
       <c r="C3" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>turnover</v>
       </c>
       <c r="D3" s="8">
@@ -1925,16 +1935,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>sales - cakes and pastries</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="7">
         <v>1200</v>
       </c>
       <c r="C4" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_income</v>
       </c>
       <c r="D4" s="8">
@@ -1945,16 +1959,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>interest received</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="7">
         <v>851200</v>
       </c>
       <c r="C5" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D5" s="8">
@@ -1965,16 +1983,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>total income</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7">
         <v>240000</v>
       </c>
       <c r="C6" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>cost_of_sales</v>
       </c>
       <c r="D6" s="8">
@@ -1985,16 +2007,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>flour and ingredients</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="7">
         <v>24000</v>
       </c>
       <c r="C7" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>cost_of_sales</v>
       </c>
       <c r="D7" s="8">
@@ -2005,16 +2031,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>packaging</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="7">
         <v>6000</v>
       </c>
       <c r="C8" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>cost_of_sales</v>
       </c>
       <c r="D8" s="8">
@@ -2025,16 +2055,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>freight inwards</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="7">
         <v>95000</v>
       </c>
       <c r="C9" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>cost_of_sales_labour</v>
       </c>
       <c r="D9" s="8">
@@ -2045,16 +2079,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>bakery wages</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="7">
         <v>365000</v>
       </c>
       <c r="C10" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D10" s="8">
@@ -2065,16 +2103,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>total cost of sales</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" s="7">
         <v>486200</v>
       </c>
       <c r="C11" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D11" s="8">
@@ -2085,16 +2127,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>gross profit</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="7">
         <v>4800</v>
       </c>
       <c r="C12" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D12" s="8">
@@ -2105,16 +2151,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>accounting fees</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="7">
         <v>3600</v>
       </c>
       <c r="C13" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D13" s="8">
@@ -2125,16 +2175,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>advertising</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="7">
         <v>1900</v>
       </c>
       <c r="C14" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D14" s="8">
@@ -2145,16 +2199,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>bank fees</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="7">
         <v>7800</v>
       </c>
       <c r="C15" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>contractor_commission</v>
       </c>
       <c r="D15" s="8">
@@ -2165,16 +2223,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>cleaning contractor</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="7">
         <v>21000</v>
       </c>
       <c r="C16" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D16" s="8">
@@ -2185,16 +2247,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>depreciation</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="7">
         <v>18000</v>
       </c>
       <c r="C17" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D17" s="8">
@@ -2205,16 +2271,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>electricity</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="7">
         <v>7400</v>
       </c>
       <c r="C18" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D18" s="8">
@@ -2225,16 +2295,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>insurance</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="7">
         <v>9500</v>
       </c>
       <c r="C19" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>motor_vehicle</v>
       </c>
       <c r="D19" s="8">
@@ -2245,16 +2319,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>motor vehicle expenses</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" s="7">
         <v>62000</v>
       </c>
       <c r="C20" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>rent</v>
       </c>
       <c r="D20" s="8">
@@ -2265,16 +2343,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>rent</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" s="7">
         <v>6200</v>
       </c>
       <c r="C21" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D21" s="8">
@@ -2285,16 +2367,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>repairs and maintenance</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="7">
         <v>175000</v>
       </c>
       <c r="C22" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>salary_wages</v>
       </c>
       <c r="D22" s="8">
@@ -2305,16 +2391,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>shop wages</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B23" s="7">
         <v>24750</v>
       </c>
       <c r="C23" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>other_expense</v>
       </c>
       <c r="D23" s="8">
@@ -2325,16 +2415,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>superannuation</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24" s="7">
         <v>45000</v>
       </c>
       <c r="C24" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>associated_persons</v>
       </c>
       <c r="D24" s="8">
@@ -2345,16 +2439,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>wages - director spouse</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25" s="7">
         <v>386950</v>
       </c>
       <c r="C25" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D25" s="8">
@@ -2365,16 +2463,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>total operating expenses</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" s="7">
         <v>99250</v>
       </c>
       <c r="C26" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D26" s="8">
@@ -2385,16 +2487,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>net profit before tax</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B27" s="7">
         <v>12000</v>
       </c>
       <c r="C27" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D27" s="8">
@@ -2405,16 +2511,20 @@
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>income tax expense</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B28" s="7">
         <v>87250</v>
       </c>
       <c r="C28" s="8" t="str">
-        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRIM(LOWER(tblPnl[[#This Row],[Account]])),tblMapping[Key],0)),"")</f>
+        <f>IFERROR(INDEX(tblMapping[Bucket],MATCH(TRUE,INDEX(tblMapping[Key]=tblPnl[[#This Row],[Key]],0),0)),"")</f>
         <v>excluded</v>
       </c>
       <c r="D28" s="8">
@@ -2424,6 +2534,10 @@
       <c r="E28" s="8">
         <f>IF(SUMPRODUCT((LOWER(TRIM(tblPnl[[#This Row],[Account]]))={"sales - bread and rolls","sales - cakes and pastries","interest received","total income","flour and ingredients","packaging","freight inwards","bakery wages","total cost of sales","gross profit","accounting fees","advertising","bank fees","cleaning contractor","depreciation","electricity","insurance","motor vehicle expenses","rent","repairs and maintenance","shop wages","superannuation","wages - director spouse","total operating expenses","net profit before tax","income tax expense","net profit"})*(tblPnl[[#This Row],[Amount]]={520000,330000,1200,851200,240000,24000,6000,95000,365000,486200,4800,3600,1900,7800,21000,18000,7400,9500,62000,6200,175000,24750,45000,386950,99250,12000,87250}))&gt;0,1,0)</f>
         <v>1</v>
+      </c>
+      <c r="F28" s="8" t="str">
+        <f>TRIM(LOWER(tblPnl[[#This Row],[Account]]))</f>
+        <v>net profit</v>
       </c>
     </row>
   </sheetData>
@@ -2454,18 +2568,18 @@
         <v>11</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>44</v>
@@ -2483,7 +2597,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>44</v>
@@ -2501,7 +2615,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>47</v>
@@ -2519,7 +2633,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>49</v>
@@ -2537,7 +2651,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>51</v>
@@ -2555,7 +2669,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>51</v>
@@ -2573,7 +2687,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>51</v>
@@ -2591,7 +2705,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>53</v>
@@ -2609,7 +2723,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>49</v>
@@ -2627,7 +2741,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>49</v>
@@ -2645,7 +2759,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>55</v>
@@ -2663,7 +2777,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>55</v>
@@ -2681,7 +2795,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>55</v>
@@ -2699,7 +2813,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>57</v>
@@ -2717,7 +2831,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>55</v>
@@ -2735,7 +2849,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>55</v>
@@ -2753,7 +2867,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>55</v>
@@ -2771,7 +2885,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>59</v>
@@ -2789,7 +2903,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>61</v>
@@ -2807,7 +2921,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>55</v>
@@ -2825,7 +2939,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>63</v>
@@ -2843,7 +2957,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B23" s="9" t="s">
         <v>55</v>
@@ -2861,7 +2975,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>66</v>
@@ -2879,7 +2993,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>49</v>
@@ -2897,7 +3011,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>49</v>
@@ -2915,7 +3029,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>49</v>
@@ -2933,7 +3047,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>49</v>
@@ -27522,7 +27636,7 @@
         <v>365</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -27732,11 +27846,11 @@
         <v>PASS</v>
       </c>
       <c r="C2" s="8">
-        <f>COUNTIFS(tblPnl[Account],"&lt;&gt;",tblPnl[Bucket],"")</f>
+        <f>SUMPRODUCT((tblPnl[Account]&lt;&gt;"")*ISNA(MATCH(tblPnl[Bucket],{"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"},0)))</f>
         <v>0</v>
       </c>
       <c r="D2" s="8" t="str">
-        <f t="array" ref="D2">IF(C2=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((tblPnl[Account]&lt;&gt;"")*(tblPnl[Bucket]="")*(ROW(tblPnl[Account])-1)))))</f>
+        <f t="array" ref="D2">IF(C2=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((tblPnl[Account]&lt;&gt;"")*ISNA(MATCH(tblPnl[Bucket],{"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"},0))*(ROW(tblPnl[Account])-1)))))</f>
         <v/>
       </c>
     </row>
@@ -27749,11 +27863,11 @@
         <v>PASS</v>
       </c>
       <c r="C3" s="8">
-        <f>COUNTIF(tblMapping[Source],"suggested")</f>
+        <f>SUMPRODUCT(--(TRIM(LOWER(tblMapping[Source]))="suggested"))</f>
         <v>0</v>
       </c>
       <c r="D3" s="8" t="str">
-        <f t="array" ref="D3">IF(C3=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((tblMapping[Source]="suggested")*(ROW(tblMapping[Account])-1)))))</f>
+        <f t="array" ref="D3">IF(C3=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((TRIM(LOWER(tblMapping[Source]))="suggested")*(ROW(tblMapping[Account])-1)))))</f>
         <v/>
       </c>
     </row>
@@ -27783,11 +27897,11 @@
         <v>PASS</v>
       </c>
       <c r="C5" s="8">
-        <f>SUMPRODUCT((COUNTIF(tblPnl[Account],tblPnl[Account])&gt;1)*(tblPnl[Account]&lt;&gt;""))</f>
+        <f>SUMPRODUCT((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((COUNTIF(tblPnl[Account],tblPnl[Account])&gt;1)*(tblPnl[Account]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
+        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Test recognised buckets by literal equality so a pasted wildcard cannot pass the benchmark bucket check
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE72EBA-8DC4-479A-968A-F3AF34DAF2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F8C752-E7C6-4F43-B097-B819F3C16655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27846,11 +27846,11 @@
         <v>PASS</v>
       </c>
       <c r="C2" s="8">
-        <f>SUMPRODUCT((tblPnl[Account]&lt;&gt;"")*ISNA(MATCH(tblPnl[Bucket],{"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"},0)))</f>
+        <f>SUMPRODUCT((tblPnl[Account]&lt;&gt;"")*(MMULT(--(tblPnl[Bucket]={"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"}),{1;1;1;1;1;1;1;1;1;1;1})=0))</f>
         <v>0</v>
       </c>
       <c r="D2" s="8" t="str">
-        <f t="array" ref="D2">IF(C2=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((tblPnl[Account]&lt;&gt;"")*ISNA(MATCH(tblPnl[Bucket],{"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"},0))*(ROW(tblPnl[Account])-1)))))</f>
+        <f t="array" ref="D2">IF(C2=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((tblPnl[Account]&lt;&gt;"")*(MMULT(--(tblPnl[Bucket]={"turnover","other_income","cost_of_sales","cost_of_sales_labour","salary_wages","contractor_commission","associated_persons","rent","motor_vehicle","other_expense","excluded"}),{1;1;1;1;1;1;1;1;1;1;1})=0)*(ROW(tblPnl[Account])-1)))))</f>
         <v/>
       </c>
     </row>

</xml_diff>